<commit_message>
add economic_moat_wide score and add new tracking data sheet
</commit_message>
<xml_diff>
--- a/etf_screener/data/top-performer-a (2).xlsx
+++ b/etf_screener/data/top-performer-a (2).xlsx
@@ -1398,7 +1398,7 @@
         <v>0.35</v>
       </c>
       <c r="D2">
-        <v>4.7534246575342465</v>
+        <v>4.772602739726028</v>
       </c>
       <c r="F2" t="s">
         <v>29</v>
@@ -1410,7 +1410,7 @@
         <v>31</v>
       </c>
       <c r="K2">
-        <v>11.758904109589041</v>
+        <v>11.778082191780822</v>
       </c>
       <c r="L2" t="s">
         <v>32</v>
@@ -1457,7 +1457,7 @@
         <v>0.36</v>
       </c>
       <c r="D3">
-        <v>14.346118721461186</v>
+        <v>14.365296803652967</v>
       </c>
       <c r="F3" t="s">
         <v>29</v>
@@ -1469,7 +1469,7 @@
         <v>35</v>
       </c>
       <c r="K3">
-        <v>19.18082191780822</v>
+        <v>19.2</v>
       </c>
       <c r="L3" t="s">
         <v>36</v>
@@ -1519,7 +1519,7 @@
         <v>0.39</v>
       </c>
       <c r="D4">
-        <v>14.346118721461186</v>
+        <v>14.365296803652967</v>
       </c>
       <c r="F4" t="s">
         <v>29</v>
@@ -1531,7 +1531,7 @@
         <v>35</v>
       </c>
       <c r="K4">
-        <v>19.18082191780822</v>
+        <v>19.2</v>
       </c>
       <c r="L4" t="s">
         <v>36</v>
@@ -1581,7 +1581,7 @@
         <v>0.35</v>
       </c>
       <c r="D5">
-        <v>7.363470319634703</v>
+        <v>7.382648401826484</v>
       </c>
       <c r="F5" t="s">
         <v>29</v>
@@ -1593,7 +1593,7 @@
         <v>39</v>
       </c>
       <c r="K5">
-        <v>11.758904109589041</v>
+        <v>11.778082191780822</v>
       </c>
       <c r="L5" t="s">
         <v>32</v>
@@ -1646,7 +1646,7 @@
         <v>0.75</v>
       </c>
       <c r="D6">
-        <v>2.116712328767123</v>
+        <v>2.135890410958904</v>
       </c>
       <c r="F6" t="s">
         <v>41</v>
@@ -1658,7 +1658,7 @@
         <v>43</v>
       </c>
       <c r="K6">
-        <v>3.23013698630137</v>
+        <v>3.249315068493151</v>
       </c>
       <c r="L6" t="s">
         <v>44</v>
@@ -1696,7 +1696,7 @@
         <v>0.4</v>
       </c>
       <c r="D7">
-        <v>7.195433789954339</v>
+        <v>7.2146118721461185</v>
       </c>
       <c r="F7" t="s">
         <v>29</v>
@@ -1708,7 +1708,7 @@
         <v>47</v>
       </c>
       <c r="K7">
-        <v>11.506849315068493</v>
+        <v>11.526027397260274</v>
       </c>
       <c r="L7" t="s">
         <v>32</v>
@@ -1752,7 +1752,7 @@
         <v>0.51</v>
       </c>
       <c r="D8">
-        <v>4.652054794520548</v>
+        <v>4.671232876712328</v>
       </c>
       <c r="F8" t="s">
         <v>41</v>
@@ -1764,7 +1764,7 @@
         <v>50</v>
       </c>
       <c r="K8">
-        <v>4.652054794520548</v>
+        <v>4.671232876712328</v>
       </c>
       <c r="L8" t="s">
         <v>51</v>
@@ -1802,7 +1802,7 @@
         <v>0.09</v>
       </c>
       <c r="D9">
-        <v>1.4493150684931506</v>
+        <v>1.4684931506849315</v>
       </c>
       <c r="F9" t="s">
         <v>29</v>
@@ -1814,7 +1814,7 @@
         <v>53</v>
       </c>
       <c r="K9">
-        <v>1.4493150684931506</v>
+        <v>1.4684931506849315</v>
       </c>
       <c r="L9" t="s">
         <v>54</v>
@@ -1864,7 +1864,7 @@
         <v>0.18</v>
       </c>
       <c r="D10">
-        <v>3.345205479452055</v>
+        <v>3.3643835616438356</v>
       </c>
       <c r="F10" t="s">
         <v>29</v>
@@ -1876,7 +1876,7 @@
         <v>56</v>
       </c>
       <c r="K10">
-        <v>3.345205479452055</v>
+        <v>3.3643835616438356</v>
       </c>
       <c r="L10" t="s">
         <v>56</v>
@@ -1917,7 +1917,7 @@
         <v>0.39</v>
       </c>
       <c r="D11">
-        <v>2.6593607305936073</v>
+        <v>2.6785388127853884</v>
       </c>
       <c r="F11" t="s">
         <v>29</v>
@@ -1929,7 +1929,7 @@
         <v>58</v>
       </c>
       <c r="K11">
-        <v>3.115068493150685</v>
+        <v>3.1342465753424658</v>
       </c>
       <c r="L11" t="s">
         <v>59</v>
@@ -1967,7 +1967,7 @@
         <v>0.09</v>
       </c>
       <c r="D12">
-        <v>1.4493150684931506</v>
+        <v>1.4684931506849315</v>
       </c>
       <c r="E12">
         <v>6.8</v>
@@ -1982,7 +1982,7 @@
         <v>61</v>
       </c>
       <c r="K12">
-        <v>1.4493150684931506</v>
+        <v>1.4684931506849315</v>
       </c>
       <c r="L12" t="s">
         <v>62</v>
@@ -2032,7 +2032,7 @@
         <v>0.29</v>
       </c>
       <c r="D13">
-        <v>5.898630136986302</v>
+        <v>5.917808219178082</v>
       </c>
       <c r="E13">
         <v>10.5</v>
@@ -2047,7 +2047,7 @@
         <v>64</v>
       </c>
       <c r="K13">
-        <v>8.775342465753425</v>
+        <v>8.794520547945206</v>
       </c>
       <c r="L13" t="s">
         <v>65</v>
@@ -2088,7 +2088,7 @@
         <v>0.08</v>
       </c>
       <c r="D14">
-        <v>4.4815068493150685</v>
+        <v>4.50068493150685</v>
       </c>
       <c r="F14" t="s">
         <v>29</v>
@@ -2100,7 +2100,7 @@
         <v>67</v>
       </c>
       <c r="K14">
-        <v>13.923287671232877</v>
+        <v>13.942465753424658</v>
       </c>
       <c r="L14" t="s">
         <v>68</v>
@@ -2188,7 +2188,7 @@
         <v>0.69</v>
       </c>
       <c r="D16">
-        <v>7.924657534246576</v>
+        <v>7.943835616438356</v>
       </c>
       <c r="F16" t="s">
         <v>41</v>
@@ -2200,7 +2200,7 @@
         <v>73</v>
       </c>
       <c r="K16">
-        <v>8.424657534246576</v>
+        <v>8.443835616438356</v>
       </c>
       <c r="L16" t="s">
         <v>74</v>
@@ -2247,7 +2247,7 @@
         <v>0.39</v>
       </c>
       <c r="D17">
-        <v>12.067579908675798</v>
+        <v>12.08675799086758</v>
       </c>
       <c r="F17" t="s">
         <v>29</v>
@@ -2259,7 +2259,7 @@
         <v>35</v>
       </c>
       <c r="K17">
-        <v>15.136986301369863</v>
+        <v>15.156164383561643</v>
       </c>
       <c r="L17" t="s">
         <v>36</v>
@@ -2309,7 +2309,7 @@
         <v>0.53</v>
       </c>
       <c r="D18">
-        <v>3.46986301369863</v>
+        <v>3.4890410958904106</v>
       </c>
       <c r="F18" t="s">
         <v>41</v>
@@ -2321,7 +2321,7 @@
         <v>78</v>
       </c>
       <c r="K18">
-        <v>5.191780821917808</v>
+        <v>5.210958904109589</v>
       </c>
       <c r="L18" t="s">
         <v>79</v>
@@ -2362,7 +2362,7 @@
         <v>0.19</v>
       </c>
       <c r="D19">
-        <v>5.142465753424657</v>
+        <v>5.161643835616438</v>
       </c>
       <c r="F19" t="s">
         <v>29</v>
@@ -2374,7 +2374,7 @@
         <v>81</v>
       </c>
       <c r="K19">
-        <v>5.142465753424657</v>
+        <v>5.161643835616438</v>
       </c>
       <c r="L19" t="s">
         <v>82</v>
@@ -2415,7 +2415,7 @@
         <v>0.15</v>
       </c>
       <c r="D20">
-        <v>3.817808219178082</v>
+        <v>3.8369863013698633</v>
       </c>
       <c r="E20">
         <v>9.5</v>
@@ -2430,7 +2430,7 @@
         <v>67</v>
       </c>
       <c r="K20">
-        <v>11.26849315068493</v>
+        <v>11.287671232876713</v>
       </c>
       <c r="L20" t="s">
         <v>68</v>
@@ -2474,7 +2474,7 @@
         <v>0.35</v>
       </c>
       <c r="D21">
-        <v>8.561643835616438</v>
+        <v>8.580821917808219</v>
       </c>
       <c r="E21">
         <v>0.2</v>
@@ -2489,7 +2489,7 @@
         <v>85</v>
       </c>
       <c r="K21">
-        <v>14.624657534246575</v>
+        <v>14.643835616438356</v>
       </c>
       <c r="L21" t="s">
         <v>86</v>
@@ -2533,7 +2533,7 @@
         <v>0.15</v>
       </c>
       <c r="D22">
-        <v>2.73972602739726</v>
+        <v>2.758904109589041</v>
       </c>
       <c r="F22" t="s">
         <v>29</v>
@@ -2545,7 +2545,7 @@
         <v>89</v>
       </c>
       <c r="K22">
-        <v>4.213698630136986</v>
+        <v>4.232876712328767</v>
       </c>
       <c r="L22" t="s">
         <v>90</v>
@@ -2583,7 +2583,7 @@
         <v>0.15</v>
       </c>
       <c r="D23">
-        <v>2.73972602739726</v>
+        <v>2.758904109589041</v>
       </c>
       <c r="F23" t="s">
         <v>29</v>
@@ -2595,7 +2595,7 @@
         <v>89</v>
       </c>
       <c r="K23">
-        <v>4.213698630136986</v>
+        <v>4.232876712328767</v>
       </c>
       <c r="L23" t="s">
         <v>90</v>
@@ -2633,7 +2633,7 @@
         <v>0.35</v>
       </c>
       <c r="D24">
-        <v>10.669863013698631</v>
+        <v>10.68904109589041</v>
       </c>
       <c r="F24" t="s">
         <v>29</v>
@@ -2645,7 +2645,7 @@
         <v>93</v>
       </c>
       <c r="K24">
-        <v>11.758904109589041</v>
+        <v>11.778082191780822</v>
       </c>
       <c r="L24" t="s">
         <v>32</v>
@@ -2698,7 +2698,7 @@
         <v>0.58</v>
       </c>
       <c r="D25">
-        <v>8.288454011741683</v>
+        <v>8.307632093933462</v>
       </c>
       <c r="F25" t="s">
         <v>29</v>
@@ -2710,7 +2710,7 @@
         <v>95</v>
       </c>
       <c r="K25">
-        <v>8.753424657534246</v>
+        <v>8.772602739726027</v>
       </c>
       <c r="L25" t="s">
         <v>96</v>
@@ -2751,7 +2751,7 @@
         <v>0.6</v>
       </c>
       <c r="D26">
-        <v>6.136986301369863</v>
+        <v>6.156164383561643</v>
       </c>
       <c r="F26" t="s">
         <v>41</v>
@@ -2763,7 +2763,7 @@
         <v>98</v>
       </c>
       <c r="K26">
-        <v>8.252054794520548</v>
+        <v>8.271232876712329</v>
       </c>
       <c r="L26" t="s">
         <v>99</v>
@@ -2804,7 +2804,7 @@
         <v>0.66</v>
       </c>
       <c r="D27">
-        <v>3.9084148727984345</v>
+        <v>3.927592954990216</v>
       </c>
       <c r="F27" t="s">
         <v>101</v>
@@ -2816,7 +2816,7 @@
         <v>102</v>
       </c>
       <c r="K27">
-        <v>4.517808219178082</v>
+        <v>4.536986301369863</v>
       </c>
       <c r="L27" t="s">
         <v>103</v>
@@ -2854,7 +2854,7 @@
         <v>0.25</v>
       </c>
       <c r="D28">
-        <v>5.754337899543379</v>
+        <v>5.77351598173516</v>
       </c>
       <c r="F28" t="s">
         <v>29</v>
@@ -2866,7 +2866,7 @@
         <v>105</v>
       </c>
       <c r="K28">
-        <v>11.758904109589041</v>
+        <v>11.778082191780822</v>
       </c>
       <c r="L28" t="s">
         <v>32</v>
@@ -2916,7 +2916,7 @@
         <v>0.45</v>
       </c>
       <c r="D29">
-        <v>5.442922374429224</v>
+        <v>5.4621004566210045</v>
       </c>
       <c r="F29" t="s">
         <v>29</v>
@@ -2928,7 +2928,7 @@
         <v>107</v>
       </c>
       <c r="K29">
-        <v>7.789041095890411</v>
+        <v>7.808219178082192</v>
       </c>
       <c r="L29" t="s">
         <v>108</v>
@@ -2969,7 +2969,7 @@
         <v>0.39</v>
       </c>
       <c r="D30">
-        <v>4.398630136986301</v>
+        <v>4.417808219178083</v>
       </c>
       <c r="F30" t="s">
         <v>29</v>
@@ -2981,7 +2981,7 @@
         <v>67</v>
       </c>
       <c r="K30">
-        <v>13.591780821917808</v>
+        <v>13.610958904109589</v>
       </c>
       <c r="L30" t="s">
         <v>68</v>
@@ -3025,7 +3025,7 @@
         <v>0.55</v>
       </c>
       <c r="D31">
-        <v>6.9082191780821915</v>
+        <v>6.927397260273973</v>
       </c>
       <c r="E31">
         <v>0.2</v>
@@ -3040,7 +3040,7 @@
         <v>112</v>
       </c>
       <c r="K31">
-        <v>8.317808219178081</v>
+        <v>8.336986301369864</v>
       </c>
       <c r="L31" t="s">
         <v>113</v>
@@ -3081,7 +3081,7 @@
         <v>0.15</v>
       </c>
       <c r="D32">
-        <v>5.802739726027397</v>
+        <v>5.821917808219179</v>
       </c>
       <c r="F32" t="s">
         <v>29</v>
@@ -3093,7 +3093,7 @@
         <v>81</v>
       </c>
       <c r="K32">
-        <v>5.802739726027397</v>
+        <v>5.821917808219178</v>
       </c>
       <c r="L32" t="s">
         <v>82</v>
@@ -3137,7 +3137,7 @@
         <v>0.25</v>
       </c>
       <c r="D33">
-        <v>6.204794520547946</v>
+        <v>6.223972602739726</v>
       </c>
       <c r="F33" t="s">
         <v>29</v>
@@ -3149,7 +3149,7 @@
         <v>116</v>
       </c>
       <c r="K33">
-        <v>10.863013698630137</v>
+        <v>10.882191780821918</v>
       </c>
       <c r="L33" t="s">
         <v>117</v>
@@ -3193,7 +3193,7 @@
         <v>0.43</v>
       </c>
       <c r="D34">
-        <v>9.265068493150684</v>
+        <v>9.284246575342467</v>
       </c>
       <c r="F34" t="s">
         <v>29</v>
@@ -3205,7 +3205,7 @@
         <v>120</v>
       </c>
       <c r="K34">
-        <v>19.115068493150684</v>
+        <v>19.134246575342466</v>
       </c>
       <c r="L34" t="s">
         <v>36</v>
@@ -3252,7 +3252,7 @@
         <v>0.55</v>
       </c>
       <c r="D35">
-        <v>5.189041095890411</v>
+        <v>5.208219178082191</v>
       </c>
       <c r="F35" t="s">
         <v>41</v>
@@ -3264,7 +3264,7 @@
         <v>122</v>
       </c>
       <c r="K35">
-        <v>5.189041095890411</v>
+        <v>5.208219178082191</v>
       </c>
       <c r="L35" t="s">
         <v>123</v>
@@ -3305,7 +3305,7 @@
         <v>0.6</v>
       </c>
       <c r="D36">
-        <v>14.346118721461186</v>
+        <v>14.365296803652967</v>
       </c>
       <c r="F36" t="s">
         <v>41</v>
@@ -3317,7 +3317,7 @@
         <v>35</v>
       </c>
       <c r="K36">
-        <v>19.18082191780822</v>
+        <v>19.2</v>
       </c>
       <c r="L36" t="s">
         <v>36</v>
@@ -3364,7 +3364,7 @@
         <v>0.33</v>
       </c>
       <c r="D37">
-        <v>3.6383561643835614</v>
+        <v>3.657534246575343</v>
       </c>
       <c r="F37" t="s">
         <v>29</v>
@@ -3376,7 +3376,7 @@
         <v>126</v>
       </c>
       <c r="K37">
-        <v>3.638356164383562</v>
+        <v>3.6575342465753424</v>
       </c>
       <c r="L37" t="s">
         <v>127</v>
@@ -3414,7 +3414,7 @@
         <v>0.55</v>
       </c>
       <c r="D38">
-        <v>3.6164383561643834</v>
+        <v>3.6356164383561644</v>
       </c>
       <c r="E38">
         <v>0.2</v>
@@ -3429,7 +3429,7 @@
         <v>129</v>
       </c>
       <c r="K38">
-        <v>3.6164383561643834</v>
+        <v>3.6356164383561644</v>
       </c>
       <c r="L38" t="s">
         <v>130</v>
@@ -3467,7 +3467,7 @@
         <v>0.47</v>
       </c>
       <c r="D39">
-        <v>7.924657534246576</v>
+        <v>7.943835616438356</v>
       </c>
       <c r="E39">
         <v>4.9</v>
@@ -3482,7 +3482,7 @@
         <v>73</v>
       </c>
       <c r="K39">
-        <v>8.424657534246576</v>
+        <v>8.443835616438356</v>
       </c>
       <c r="L39" t="s">
         <v>74</v>
@@ -3526,7 +3526,7 @@
         <v>0.79</v>
       </c>
       <c r="D40">
-        <v>6.841095890410959</v>
+        <v>6.86027397260274</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -3541,7 +3541,7 @@
         <v>134</v>
       </c>
       <c r="K40">
-        <v>6.841095890410959</v>
+        <v>6.86027397260274</v>
       </c>
       <c r="L40" t="s">
         <v>135</v>
@@ -3582,7 +3582,7 @@
         <v>0.21</v>
       </c>
       <c r="D41">
-        <v>11.008219178082193</v>
+        <v>11.027397260273974</v>
       </c>
       <c r="F41" t="s">
         <v>29</v>
@@ -3594,7 +3594,7 @@
         <v>137</v>
       </c>
       <c r="K41">
-        <v>17.50958904109589</v>
+        <v>17.528767123287672</v>
       </c>
       <c r="L41" t="s">
         <v>138</v>
@@ -3644,7 +3644,7 @@
         <v>0.2</v>
       </c>
       <c r="D42">
-        <v>10.127397260273973</v>
+        <v>10.146575342465752</v>
       </c>
       <c r="F42" t="s">
         <v>29</v>
@@ -3656,7 +3656,7 @@
         <v>93</v>
       </c>
       <c r="K42">
-        <v>10.673972602739726</v>
+        <v>10.693150684931506</v>
       </c>
       <c r="L42" t="s">
         <v>32</v>
@@ -3700,7 +3700,7 @@
         <v>0.77</v>
       </c>
       <c r="D43">
-        <v>3.96986301369863</v>
+        <v>3.989041095890411</v>
       </c>
       <c r="F43" t="s">
         <v>29</v>
@@ -3712,7 +3712,7 @@
         <v>142</v>
       </c>
       <c r="K43">
-        <v>4.208219178082191</v>
+        <v>4.227397260273973</v>
       </c>
       <c r="L43" t="s">
         <v>143</v>
@@ -3753,7 +3753,7 @@
         <v>0.74</v>
       </c>
       <c r="D44">
-        <v>1.9232876712328766</v>
+        <v>1.9424657534246577</v>
       </c>
       <c r="F44" t="s">
         <v>41</v>
@@ -3765,7 +3765,7 @@
         <v>145</v>
       </c>
       <c r="K44">
-        <v>3.4246575342465753</v>
+        <v>3.4438356164383563</v>
       </c>
       <c r="L44" t="s">
         <v>146</v>
@@ -3803,7 +3803,7 @@
         <v>0.3</v>
       </c>
       <c r="D45">
-        <v>3.4068493150684933</v>
+        <v>3.426027397260274</v>
       </c>
       <c r="F45" t="s">
         <v>29</v>
@@ -3821,7 +3821,7 @@
         <v>149</v>
       </c>
       <c r="K45">
-        <v>6.7534246575342465</v>
+        <v>6.772602739726027</v>
       </c>
       <c r="L45" t="s">
         <v>150</v>
@@ -3871,7 +3871,7 @@
         <v>0.09</v>
       </c>
       <c r="D46">
-        <v>4.4664383561643834</v>
+        <v>4.485616438356164</v>
       </c>
       <c r="E46">
         <v>5.2</v>
@@ -3886,7 +3886,7 @@
         <v>152</v>
       </c>
       <c r="K46">
-        <v>6.32054794520548</v>
+        <v>6.33972602739726</v>
       </c>
       <c r="L46" t="s">
         <v>153</v>
@@ -3927,7 +3927,7 @@
         <v>0.35</v>
       </c>
       <c r="D47">
-        <v>7.363470319634704</v>
+        <v>7.382648401826483</v>
       </c>
       <c r="F47" t="s">
         <v>29</v>
@@ -3939,7 +3939,7 @@
         <v>155</v>
       </c>
       <c r="K47">
-        <v>11.758904109589041</v>
+        <v>11.778082191780822</v>
       </c>
       <c r="L47" t="s">
         <v>32</v>
@@ -3989,7 +3989,7 @@
         <v>0.35</v>
       </c>
       <c r="D48">
-        <v>2.9986301369863013</v>
+        <v>3.0178082191780824</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -4004,7 +4004,7 @@
         <v>157</v>
       </c>
       <c r="K48">
-        <v>4.249315068493151</v>
+        <v>4.2684931506849315</v>
       </c>
       <c r="L48" t="s">
         <v>158</v>
@@ -4022,16 +4022,16 @@
         <v>9.32044</v>
       </c>
       <c r="U48">
-        <v>4.19</v>
+        <v>4.25</v>
       </c>
       <c r="V48">
-        <v>4.32</v>
+        <v>4.38</v>
       </c>
       <c r="W48">
-        <v>4.17</v>
+        <v>4.21</v>
       </c>
       <c r="AB48">
-        <v>1.85</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.25">
@@ -4042,7 +4042,7 @@
         <v>0.38</v>
       </c>
       <c r="D49">
-        <v>4.4815068493150685</v>
+        <v>4.50068493150685</v>
       </c>
       <c r="F49" t="s">
         <v>29</v>
@@ -4054,7 +4054,7 @@
         <v>67</v>
       </c>
       <c r="K49">
-        <v>13.923287671232877</v>
+        <v>13.942465753424658</v>
       </c>
       <c r="L49" t="s">
         <v>68</v>
@@ -4104,7 +4104,7 @@
         <v>0.38</v>
       </c>
       <c r="D50">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F50" t="s">
         <v>29</v>
@@ -4116,7 +4116,7 @@
         <v>67</v>
       </c>
       <c r="K50">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L50" t="s">
         <v>68</v>
@@ -4166,7 +4166,7 @@
         <v>0.18</v>
       </c>
       <c r="D51">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F51" t="s">
         <v>29</v>
@@ -4178,7 +4178,7 @@
         <v>67</v>
       </c>
       <c r="K51">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L51" t="s">
         <v>68</v>
@@ -4228,7 +4228,7 @@
         <v>0.03</v>
       </c>
       <c r="D52">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F52" t="s">
         <v>29</v>
@@ -4240,7 +4240,7 @@
         <v>67</v>
       </c>
       <c r="K52">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L52" t="s">
         <v>68</v>
@@ -4290,7 +4290,7 @@
         <v>0.04</v>
       </c>
       <c r="D53">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F53" t="s">
         <v>29</v>
@@ -4302,7 +4302,7 @@
         <v>67</v>
       </c>
       <c r="K53">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L53" t="s">
         <v>68</v>
@@ -4352,7 +4352,7 @@
         <v>0.31</v>
       </c>
       <c r="D54">
-        <v>2.341095890410959</v>
+        <v>2.36027397260274</v>
       </c>
       <c r="F54" t="s">
         <v>29</v>
@@ -4364,7 +4364,7 @@
         <v>67</v>
       </c>
       <c r="K54">
-        <v>5.361643835616438</v>
+        <v>5.380821917808219</v>
       </c>
       <c r="L54" t="s">
         <v>68</v>
@@ -4405,7 +4405,7 @@
         <v>0.4</v>
       </c>
       <c r="D55">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F55" t="s">
         <v>29</v>
@@ -4417,7 +4417,7 @@
         <v>67</v>
       </c>
       <c r="K55">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L55" t="s">
         <v>68</v>
@@ -4467,7 +4467,7 @@
         <v>0.06</v>
       </c>
       <c r="D56">
-        <v>4.4815068493150685</v>
+        <v>4.50068493150685</v>
       </c>
       <c r="E56">
         <v>9.5</v>
@@ -4482,7 +4482,7 @@
         <v>67</v>
       </c>
       <c r="K56">
-        <v>13.923287671232877</v>
+        <v>13.942465753424658</v>
       </c>
       <c r="L56" t="s">
         <v>68</v>
@@ -4532,7 +4532,7 @@
         <v>0.16</v>
       </c>
       <c r="D57">
-        <v>4.502739726027397</v>
+        <v>4.521917808219178</v>
       </c>
       <c r="F57" t="s">
         <v>29</v>
@@ -4544,7 +4544,7 @@
         <v>67</v>
       </c>
       <c r="K57">
-        <v>14.008219178082191</v>
+        <v>14.027397260273972</v>
       </c>
       <c r="L57" t="s">
         <v>68</v>
@@ -4594,7 +4594,7 @@
         <v>0.3</v>
       </c>
       <c r="D58">
-        <v>3.0842465753424655</v>
+        <v>3.103424657534246</v>
       </c>
       <c r="F58" t="s">
         <v>29</v>
@@ -4606,7 +4606,7 @@
         <v>67</v>
       </c>
       <c r="K58">
-        <v>8.334246575342465</v>
+        <v>8.353424657534246</v>
       </c>
       <c r="L58" t="s">
         <v>68</v>
@@ -4647,7 +4647,7 @@
         <v>0.29</v>
       </c>
       <c r="D59">
-        <v>9.273287671232877</v>
+        <v>9.292465753424658</v>
       </c>
       <c r="F59" t="s">
         <v>29</v>
@@ -4659,7 +4659,7 @@
         <v>120</v>
       </c>
       <c r="K59">
-        <v>19.147945205479452</v>
+        <v>19.167123287671235</v>
       </c>
       <c r="L59" t="s">
         <v>36</v>
@@ -4706,7 +4706,7 @@
         <v>0.4</v>
       </c>
       <c r="D60">
-        <v>5.736301369863014</v>
+        <v>5.755479452054795</v>
       </c>
       <c r="F60" t="s">
         <v>29</v>
@@ -4724,7 +4724,7 @@
         <v>173</v>
       </c>
       <c r="K60">
-        <v>11.183561643835617</v>
+        <v>11.202739726027398</v>
       </c>
       <c r="L60" t="s">
         <v>174</v>
@@ -4806,7 +4806,7 @@
         <v>0.37</v>
       </c>
       <c r="D62">
-        <v>4.4815068493150685</v>
+        <v>4.50068493150685</v>
       </c>
       <c r="F62" t="s">
         <v>29</v>
@@ -4818,7 +4818,7 @@
         <v>67</v>
       </c>
       <c r="K62">
-        <v>13.923287671232877</v>
+        <v>13.942465753424658</v>
       </c>
       <c r="L62" t="s">
         <v>68</v>
@@ -4868,7 +4868,7 @@
         <v>0.43</v>
       </c>
       <c r="D63">
-        <v>5.715068493150685</v>
+        <v>5.734246575342466</v>
       </c>
       <c r="E63">
         <v>9.5</v>
@@ -4883,7 +4883,7 @@
         <v>178</v>
       </c>
       <c r="K63">
-        <v>11.098630136986301</v>
+        <v>11.117808219178082</v>
       </c>
       <c r="L63" t="s">
         <v>179</v>
@@ -4927,7 +4927,7 @@
         <v>0.68</v>
       </c>
       <c r="D64">
-        <v>1.4191780821917808</v>
+        <v>1.4383561643835616</v>
       </c>
       <c r="E64">
         <v>5</v>
@@ -4942,7 +4942,7 @@
         <v>181</v>
       </c>
       <c r="K64">
-        <v>1.4191780821917808</v>
+        <v>1.4383561643835616</v>
       </c>
       <c r="L64" t="s">
         <v>182</v>
@@ -4980,7 +4980,7 @@
         <v>0.53</v>
       </c>
       <c r="D65">
-        <v>6.201369863013699</v>
+        <v>6.22054794520548</v>
       </c>
       <c r="F65" t="s">
         <v>41</v>
@@ -4992,7 +4992,7 @@
         <v>178</v>
       </c>
       <c r="K65">
-        <v>12.07123287671233</v>
+        <v>12.09041095890411</v>
       </c>
       <c r="L65" t="s">
         <v>179</v>
@@ -5036,7 +5036,7 @@
         <v>0.49</v>
       </c>
       <c r="D66">
-        <v>6.419178082191781</v>
+        <v>6.438356164383562</v>
       </c>
       <c r="E66">
         <v>9.5</v>
@@ -5051,7 +5051,7 @@
         <v>178</v>
       </c>
       <c r="K66">
-        <v>12.506849315068493</v>
+        <v>12.526027397260274</v>
       </c>
       <c r="L66" t="s">
         <v>179</v>
@@ -5095,7 +5095,7 @@
         <v>0.35</v>
       </c>
       <c r="D67">
-        <v>6.419178082191781</v>
+        <v>6.438356164383562</v>
       </c>
       <c r="E67">
         <v>9.5</v>
@@ -5110,7 +5110,7 @@
         <v>178</v>
       </c>
       <c r="K67">
-        <v>12.506849315068493</v>
+        <v>12.526027397260274</v>
       </c>
       <c r="L67" t="s">
         <v>179</v>
@@ -5154,7 +5154,7 @@
         <v>0.72</v>
       </c>
       <c r="D68">
-        <v>6.097260273972603</v>
+        <v>6.116438356164384</v>
       </c>
       <c r="F68" t="s">
         <v>41</v>
@@ -5166,7 +5166,7 @@
         <v>178</v>
       </c>
       <c r="K68">
-        <v>11.863013698630137</v>
+        <v>11.882191780821918</v>
       </c>
       <c r="L68" t="s">
         <v>179</v>
@@ -5210,7 +5210,7 @@
         <v>0.35</v>
       </c>
       <c r="D69">
-        <v>5.715068493150685</v>
+        <v>5.734246575342466</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -5225,7 +5225,7 @@
         <v>178</v>
       </c>
       <c r="K69">
-        <v>11.098630136986301</v>
+        <v>11.117808219178082</v>
       </c>
       <c r="L69" t="s">
         <v>179</v>
@@ -5272,7 +5272,7 @@
         <v>0.66</v>
       </c>
       <c r="D70">
-        <v>7.157534246575342</v>
+        <v>7.176712328767123</v>
       </c>
       <c r="F70" t="s">
         <v>41</v>
@@ -5284,7 +5284,7 @@
         <v>192</v>
       </c>
       <c r="K70">
-        <v>12.4</v>
+        <v>12.419178082191781</v>
       </c>
       <c r="L70" t="s">
         <v>193</v>
@@ -5331,7 +5331,7 @@
         <v>0.25</v>
       </c>
       <c r="D71">
-        <v>3.33972602739726</v>
+        <v>3.358904109589041</v>
       </c>
       <c r="F71" t="s">
         <v>29</v>
@@ -5343,7 +5343,7 @@
         <v>195</v>
       </c>
       <c r="K71">
-        <v>4.383561643835616</v>
+        <v>4.402739726027397</v>
       </c>
       <c r="L71" t="s">
         <v>196</v>
@@ -5419,7 +5419,7 @@
         <v>0.2</v>
       </c>
       <c r="D73">
-        <v>4.383561643835616</v>
+        <v>4.402739726027397</v>
       </c>
       <c r="E73">
         <v>4.5</v>
@@ -5434,7 +5434,7 @@
         <v>200</v>
       </c>
       <c r="K73">
-        <v>4.383561643835616</v>
+        <v>4.402739726027397</v>
       </c>
       <c r="L73" t="s">
         <v>201</v>
@@ -5472,7 +5472,7 @@
         <v>0.1</v>
       </c>
       <c r="D74">
-        <v>3.578082191780822</v>
+        <v>3.5972602739726027</v>
       </c>
       <c r="F74" t="s">
         <v>29</v>
@@ -5484,7 +5484,7 @@
         <v>203</v>
       </c>
       <c r="K74">
-        <v>3.578082191780822</v>
+        <v>3.5972602739726027</v>
       </c>
       <c r="L74" t="s">
         <v>203</v>
@@ -5522,7 +5522,7 @@
         <v>0.15</v>
       </c>
       <c r="D75">
-        <v>2.6383561643835614</v>
+        <v>2.6575342465753424</v>
       </c>
       <c r="F75" t="s">
         <v>29</v>
@@ -5534,7 +5534,7 @@
         <v>67</v>
       </c>
       <c r="K75">
-        <v>6.550684931506849</v>
+        <v>6.5698630136986305</v>
       </c>
       <c r="L75" t="s">
         <v>68</v>
@@ -5575,7 +5575,7 @@
         <v>0.65</v>
       </c>
       <c r="D76">
-        <v>3.367123287671233</v>
+        <v>3.3863013698630136</v>
       </c>
       <c r="F76" t="s">
         <v>29</v>
@@ -5587,7 +5587,7 @@
         <v>206</v>
       </c>
       <c r="K76">
-        <v>3.367123287671233</v>
+        <v>3.3863013698630136</v>
       </c>
       <c r="L76" t="s">
         <v>206</v>
@@ -5625,7 +5625,7 @@
         <v>0.084</v>
       </c>
       <c r="D77">
-        <v>4.4089041095890416</v>
+        <v>4.428082191780822</v>
       </c>
       <c r="F77" t="s">
         <v>29</v>
@@ -5637,7 +5637,7 @@
         <v>208</v>
       </c>
       <c r="K77">
-        <v>12.786301369863013</v>
+        <v>12.805479452054794</v>
       </c>
       <c r="L77" t="s">
         <v>68</v>
@@ -5681,7 +5681,7 @@
         <v>0.6</v>
       </c>
       <c r="D78">
-        <v>5.4301369863013695</v>
+        <v>5.449315068493151</v>
       </c>
       <c r="F78" t="s">
         <v>29</v>
@@ -5693,7 +5693,7 @@
         <v>210</v>
       </c>
       <c r="K78">
-        <v>5.4301369863013695</v>
+        <v>5.449315068493151</v>
       </c>
       <c r="L78" t="s">
         <v>210</v>
@@ -5737,7 +5737,7 @@
         <v>0.23</v>
       </c>
       <c r="D79">
-        <v>7.175342465753425</v>
+        <v>7.1945205479452055</v>
       </c>
       <c r="E79">
         <v>8.4</v>
@@ -5752,7 +5752,7 @@
         <v>212</v>
       </c>
       <c r="K79">
-        <v>11.843835616438357</v>
+        <v>11.863013698630137</v>
       </c>
       <c r="L79" t="s">
         <v>213</v>
@@ -5799,7 +5799,7 @@
         <v>0.19</v>
       </c>
       <c r="D80">
-        <v>5.8561643835616435</v>
+        <v>5.875342465753425</v>
       </c>
       <c r="F80" t="s">
         <v>29</v>
@@ -5811,7 +5811,7 @@
         <v>215</v>
       </c>
       <c r="K80">
-        <v>8.75068493150685</v>
+        <v>8.76986301369863</v>
       </c>
       <c r="L80" t="s">
         <v>216</v>
@@ -5852,7 +5852,7 @@
         <v>0.25</v>
       </c>
       <c r="D81">
-        <v>3.063013698630137</v>
+        <v>3.0821917808219177</v>
       </c>
       <c r="F81" t="s">
         <v>29</v>
@@ -5864,7 +5864,7 @@
         <v>218</v>
       </c>
       <c r="K81">
-        <v>3.063013698630137</v>
+        <v>3.0821917808219177</v>
       </c>
       <c r="L81" t="s">
         <v>51</v>
@@ -5899,7 +5899,7 @@
         <v>0.09</v>
       </c>
       <c r="D82">
-        <v>5.856164383561644</v>
+        <v>5.875342465753425</v>
       </c>
       <c r="F82" t="s">
         <v>29</v>
@@ -5911,7 +5911,7 @@
         <v>215</v>
       </c>
       <c r="K82">
-        <v>8.75068493150685</v>
+        <v>8.76986301369863</v>
       </c>
       <c r="L82" t="s">
         <v>216</v>
@@ -5952,7 +5952,7 @@
         <v>0.18</v>
       </c>
       <c r="D83">
-        <v>7.930410958904109</v>
+        <v>7.949589041095891</v>
       </c>
       <c r="F83" t="s">
         <v>29</v>
@@ -5964,7 +5964,7 @@
         <v>221</v>
       </c>
       <c r="K83">
-        <v>8.545205479452054</v>
+        <v>8.564383561643835</v>
       </c>
       <c r="L83" t="s">
         <v>222</v>
@@ -6005,7 +6005,7 @@
         <v>0.084</v>
       </c>
       <c r="D84">
-        <v>4.4089041095890416</v>
+        <v>4.428082191780822</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -6020,7 +6020,7 @@
         <v>208</v>
       </c>
       <c r="K84">
-        <v>12.786301369863013</v>
+        <v>12.805479452054794</v>
       </c>
       <c r="L84" t="s">
         <v>68</v>
@@ -6099,7 +6099,7 @@
         <v>0.55</v>
       </c>
       <c r="D86">
-        <v>15.63013698630137</v>
+        <v>15.649315068493152</v>
       </c>
       <c r="F86" t="s">
         <v>29</v>
@@ -6111,7 +6111,7 @@
         <v>95</v>
       </c>
       <c r="K86">
-        <v>18.706849315068492</v>
+        <v>18.726027397260275</v>
       </c>
       <c r="L86" t="s">
         <v>96</v>
@@ -6158,7 +6158,7 @@
         <v>0.43</v>
       </c>
       <c r="D87">
-        <v>4.4739726027397255</v>
+        <v>4.493150684931507</v>
       </c>
       <c r="F87" t="s">
         <v>29</v>
@@ -6170,7 +6170,7 @@
         <v>227</v>
       </c>
       <c r="K87">
-        <v>5.495890410958904</v>
+        <v>5.515068493150685</v>
       </c>
       <c r="L87" t="s">
         <v>228</v>
@@ -6211,7 +6211,7 @@
         <v>0.38</v>
       </c>
       <c r="D88">
-        <v>2.43013698630137</v>
+        <v>2.4493150684931506</v>
       </c>
       <c r="F88" t="s">
         <v>29</v>
@@ -6229,7 +6229,7 @@
         <v>231</v>
       </c>
       <c r="K88">
-        <v>2.43013698630137</v>
+        <v>2.4493150684931506</v>
       </c>
       <c r="L88" t="s">
         <v>228</v>
@@ -6273,7 +6273,7 @@
         <v>0.74</v>
       </c>
       <c r="D89">
-        <v>1.9602739726027396</v>
+        <v>1.9794520547945207</v>
       </c>
       <c r="F89" t="s">
         <v>41</v>
@@ -6285,7 +6285,7 @@
         <v>145</v>
       </c>
       <c r="K89">
-        <v>3.4986301369863013</v>
+        <v>3.5178082191780824</v>
       </c>
       <c r="L89" t="s">
         <v>146</v>
@@ -6323,7 +6323,7 @@
         <v>0.56</v>
       </c>
       <c r="D90">
-        <v>15.798434442270059</v>
+        <v>15.81761252446184</v>
       </c>
       <c r="F90" t="s">
         <v>101</v>
@@ -6335,7 +6335,7 @@
         <v>95</v>
       </c>
       <c r="K90">
-        <v>18.942465753424656</v>
+        <v>18.96164383561644</v>
       </c>
       <c r="L90" t="s">
         <v>96</v>
@@ -6385,7 +6385,7 @@
         <v>0.55</v>
       </c>
       <c r="D91">
-        <v>16.604696673189824</v>
+        <v>16.623874755381603</v>
       </c>
       <c r="E91">
         <v>2.9</v>
@@ -6400,7 +6400,7 @@
         <v>235</v>
       </c>
       <c r="K91">
-        <v>20.13150684931507</v>
+        <v>20.15068493150685</v>
       </c>
       <c r="L91" t="s">
         <v>236</v>
@@ -6450,7 +6450,7 @@
         <v>0.59</v>
       </c>
       <c r="D92">
-        <v>4.398630136986301</v>
+        <v>4.417808219178083</v>
       </c>
       <c r="F92" t="s">
         <v>29</v>
@@ -6462,7 +6462,7 @@
         <v>67</v>
       </c>
       <c r="K92">
-        <v>13.591780821917808</v>
+        <v>13.610958904109589</v>
       </c>
       <c r="L92" t="s">
         <v>68</v>
@@ -6512,7 +6512,7 @@
         <v>0.5</v>
       </c>
       <c r="D93">
-        <v>4.398630136986301</v>
+        <v>4.417808219178083</v>
       </c>
       <c r="F93" t="s">
         <v>41</v>
@@ -6524,7 +6524,7 @@
         <v>67</v>
       </c>
       <c r="K93">
-        <v>13.591780821917808</v>
+        <v>13.610958904109589</v>
       </c>
       <c r="L93" t="s">
         <v>68</v>
@@ -6574,7 +6574,7 @@
         <v>0.15</v>
       </c>
       <c r="D94">
-        <v>2.8541095890410957</v>
+        <v>2.8732876712328768</v>
       </c>
       <c r="F94" t="s">
         <v>29</v>
@@ -6586,7 +6586,7 @@
         <v>67</v>
       </c>
       <c r="K94">
-        <v>7.413698630136986</v>
+        <v>7.432876712328767</v>
       </c>
       <c r="L94" t="s">
         <v>68</v>
@@ -6627,7 +6627,7 @@
         <v>0.5</v>
       </c>
       <c r="D95">
-        <v>4.398630136986301</v>
+        <v>4.417808219178083</v>
       </c>
       <c r="E95">
         <v>9.5</v>
@@ -6642,7 +6642,7 @@
         <v>67</v>
       </c>
       <c r="K95">
-        <v>13.591780821917808</v>
+        <v>13.610958904109589</v>
       </c>
       <c r="L95" t="s">
         <v>68</v>
@@ -6692,7 +6692,7 @@
         <v>0.49</v>
       </c>
       <c r="D96">
-        <v>4.419178082191781</v>
+        <v>4.438356164383562</v>
       </c>
       <c r="F96" t="s">
         <v>41</v>
@@ -6704,7 +6704,7 @@
         <v>67</v>
       </c>
       <c r="K96">
-        <v>13.673972602739726</v>
+        <v>13.693150684931506</v>
       </c>
       <c r="L96" t="s">
         <v>68</v>
@@ -6751,7 +6751,7 @@
         <v>0.55</v>
       </c>
       <c r="D97">
-        <v>5.147945205479452</v>
+        <v>5.167123287671233</v>
       </c>
       <c r="F97" t="s">
         <v>41</v>
@@ -6763,7 +6763,7 @@
         <v>85</v>
       </c>
       <c r="K97">
-        <v>7.7972602739726025</v>
+        <v>7.816438356164384</v>
       </c>
       <c r="L97" t="s">
         <v>86</v>
@@ -6807,7 +6807,7 @@
         <v>0.42</v>
       </c>
       <c r="D98">
-        <v>7.511415525114155</v>
+        <v>7.530593607305936</v>
       </c>
       <c r="F98" t="s">
         <v>29</v>
@@ -6819,7 +6819,7 @@
         <v>244</v>
       </c>
       <c r="K98">
-        <v>10.057534246575342</v>
+        <v>10.076712328767123</v>
       </c>
       <c r="L98" t="s">
         <v>117</v>
@@ -6863,7 +6863,7 @@
         <v>0.59</v>
       </c>
       <c r="D99">
-        <v>4.398630136986301</v>
+        <v>4.417808219178083</v>
       </c>
       <c r="F99" t="s">
         <v>101</v>
@@ -6875,7 +6875,7 @@
         <v>67</v>
       </c>
       <c r="K99">
-        <v>13.591780821917808</v>
+        <v>13.610958904109589</v>
       </c>
       <c r="L99" t="s">
         <v>68</v>
@@ -6922,7 +6922,7 @@
         <v>0.35</v>
       </c>
       <c r="D100">
-        <v>6.8410958904109584</v>
+        <v>6.86027397260274</v>
       </c>
       <c r="F100" t="s">
         <v>29</v>
@@ -6934,7 +6934,7 @@
         <v>247</v>
       </c>
       <c r="K100">
-        <v>11.345205479452055</v>
+        <v>11.364383561643836</v>
       </c>
       <c r="L100" t="s">
         <v>248</v>
@@ -6978,7 +6978,7 @@
         <v>0.5</v>
       </c>
       <c r="D101">
-        <v>5.764383561643836</v>
+        <v>5.7835616438356166</v>
       </c>
       <c r="F101" t="s">
         <v>41</v>
@@ -6990,7 +6990,7 @@
         <v>50</v>
       </c>
       <c r="K101">
-        <v>5.764383561643836</v>
+        <v>5.7835616438356166</v>
       </c>
       <c r="L101" t="s">
         <v>51</v>
@@ -7031,7 +7031,7 @@
         <v>0.05</v>
       </c>
       <c r="D102">
-        <v>3.1849315068493147</v>
+        <v>3.2041095890410958</v>
       </c>
       <c r="F102" t="s">
         <v>29</v>
@@ -7043,7 +7043,7 @@
         <v>67</v>
       </c>
       <c r="K102">
-        <v>8.736986301369862</v>
+        <v>8.756164383561643</v>
       </c>
       <c r="L102" t="s">
         <v>68</v>
@@ -7084,7 +7084,7 @@
         <v>0.42</v>
       </c>
       <c r="D103">
-        <v>3.6267123287671232</v>
+        <v>3.645890410958904</v>
       </c>
       <c r="F103" t="s">
         <v>29</v>
@@ -7096,7 +7096,7 @@
         <v>252</v>
       </c>
       <c r="K103">
-        <v>4.361643835616438</v>
+        <v>4.380821917808219</v>
       </c>
       <c r="L103" t="s">
         <v>253</v>
@@ -7134,7 +7134,7 @@
         <v>0.09</v>
       </c>
       <c r="D104">
-        <v>7.094063926940639</v>
+        <v>7.113242009132421</v>
       </c>
       <c r="E104">
         <v>11.6</v>
@@ -7149,7 +7149,7 @@
         <v>255</v>
       </c>
       <c r="K104">
-        <v>14.432876712328767</v>
+        <v>14.452054794520548</v>
       </c>
       <c r="L104" t="s">
         <v>256</v>
@@ -7199,7 +7199,7 @@
         <v>0.3</v>
       </c>
       <c r="D105">
-        <v>4.438356164383562</v>
+        <v>4.457534246575342</v>
       </c>
       <c r="F105" t="s">
         <v>29</v>
@@ -7211,7 +7211,7 @@
         <v>258</v>
       </c>
       <c r="K105">
-        <v>4.438356164383562</v>
+        <v>4.457534246575342</v>
       </c>
       <c r="L105" t="s">
         <v>259</v>
@@ -7249,7 +7249,7 @@
         <v>0.27</v>
       </c>
       <c r="D106">
-        <v>6.676027397260274</v>
+        <v>6.6952054794520555</v>
       </c>
       <c r="F106" t="s">
         <v>29</v>
@@ -7261,7 +7261,7 @@
         <v>261</v>
       </c>
       <c r="K106">
-        <v>16.432876712328767</v>
+        <v>16.45205479452055</v>
       </c>
       <c r="L106" t="s">
         <v>256</v>
@@ -7311,7 +7311,7 @@
         <v>0.35</v>
       </c>
       <c r="D107">
-        <v>5.984246575342466</v>
+        <v>6.0034246575342465</v>
       </c>
       <c r="F107" t="s">
         <v>29</v>
@@ -7323,7 +7323,7 @@
         <v>263</v>
       </c>
       <c r="K107">
-        <v>9.652054794520549</v>
+        <v>9.67123287671233</v>
       </c>
       <c r="L107" t="s">
         <v>264</v>
@@ -7370,7 +7370,7 @@
         <v>0.15</v>
       </c>
       <c r="D108">
-        <v>2.6965753424657533</v>
+        <v>2.7157534246575343</v>
       </c>
       <c r="F108" t="s">
         <v>29</v>
@@ -7382,7 +7382,7 @@
         <v>152</v>
       </c>
       <c r="K108">
-        <v>3.0575342465753423</v>
+        <v>3.0767123287671234</v>
       </c>
       <c r="L108" t="s">
         <v>153</v>
@@ -7417,7 +7417,7 @@
         <v>0.6</v>
       </c>
       <c r="D109">
-        <v>5.7</v>
+        <v>5.719178082191781</v>
       </c>
       <c r="F109" t="s">
         <v>29</v>
@@ -7429,7 +7429,7 @@
         <v>267</v>
       </c>
       <c r="K109">
-        <v>7.254794520547946</v>
+        <v>7.273972602739726</v>
       </c>
       <c r="L109" t="s">
         <v>268</v>
@@ -7473,7 +7473,7 @@
         <v>0.95</v>
       </c>
       <c r="D110">
-        <v>3.778082191780822</v>
+        <v>3.7972602739726025</v>
       </c>
       <c r="F110" t="s">
         <v>70</v>
@@ -7485,7 +7485,7 @@
         <v>270</v>
       </c>
       <c r="K110">
-        <v>5.978082191780822</v>
+        <v>5.997260273972603</v>
       </c>
       <c r="L110" t="s">
         <v>271</v>
@@ -7529,7 +7529,7 @@
         <v>0.89</v>
       </c>
       <c r="D111">
-        <v>3.65296803652968</v>
+        <v>3.6721461187214612</v>
       </c>
       <c r="F111" t="s">
         <v>101</v>
@@ -7541,7 +7541,7 @@
         <v>273</v>
       </c>
       <c r="K111">
-        <v>4.47945205479452</v>
+        <v>4.498630136986302</v>
       </c>
       <c r="L111" t="s">
         <v>274</v>
@@ -7579,7 +7579,7 @@
         <v>0.04</v>
       </c>
       <c r="D112">
-        <v>5.767123287671233</v>
+        <v>5.786301369863014</v>
       </c>
       <c r="E112">
         <v>8.7</v>
@@ -7594,7 +7594,7 @@
         <v>200</v>
       </c>
       <c r="K112">
-        <v>5.767123287671233</v>
+        <v>5.786301369863014</v>
       </c>
       <c r="L112" t="s">
         <v>201</v>
@@ -7635,7 +7635,7 @@
         <v>0.11</v>
       </c>
       <c r="D113">
-        <v>4.526712328767124</v>
+        <v>4.545890410958904</v>
       </c>
       <c r="F113" t="s">
         <v>29</v>
@@ -7647,7 +7647,7 @@
         <v>277</v>
       </c>
       <c r="K113">
-        <v>8.134246575342466</v>
+        <v>8.153424657534247</v>
       </c>
       <c r="L113" t="s">
         <v>278</v>
@@ -7688,7 +7688,7 @@
         <v>0.19</v>
       </c>
       <c r="D114">
-        <v>4.454109589041096</v>
+        <v>4.473287671232876</v>
       </c>
       <c r="F114" t="s">
         <v>29</v>
@@ -7700,7 +7700,7 @@
         <v>277</v>
       </c>
       <c r="K114">
-        <v>7.989041095890411</v>
+        <v>8.008219178082191</v>
       </c>
       <c r="L114" t="s">
         <v>278</v>
@@ -7718,16 +7718,16 @@
         <v>30.76263</v>
       </c>
       <c r="U114">
-        <v>0.77</v>
+        <v>0.68</v>
       </c>
       <c r="V114">
-        <v>0.84</v>
+        <v>0.76</v>
       </c>
       <c r="W114">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="X114">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="AB114">
         <v>0.3</v>
@@ -7776,7 +7776,7 @@
         <v>0.25</v>
       </c>
       <c r="D116">
-        <v>6.002739726027397</v>
+        <v>6.021917808219178</v>
       </c>
       <c r="F116" t="s">
         <v>29</v>
@@ -7788,7 +7788,7 @@
         <v>282</v>
       </c>
       <c r="K116">
-        <v>6.857534246575343</v>
+        <v>6.876712328767123</v>
       </c>
       <c r="L116" t="s">
         <v>283</v>
@@ -7829,7 +7829,7 @@
         <v>0.31</v>
       </c>
       <c r="D117">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="E117">
         <v>0.2</v>
@@ -7844,7 +7844,7 @@
         <v>285</v>
       </c>
       <c r="K117">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="L117" t="s">
         <v>283</v>
@@ -7882,7 +7882,7 @@
         <v>0.21</v>
       </c>
       <c r="D118">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="F118" t="s">
         <v>29</v>
@@ -7894,7 +7894,7 @@
         <v>285</v>
       </c>
       <c r="K118">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="L118" t="s">
         <v>283</v>
@@ -7932,7 +7932,7 @@
         <v>0.26</v>
       </c>
       <c r="D119">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="E119">
         <v>4.4</v>
@@ -7947,7 +7947,7 @@
         <v>285</v>
       </c>
       <c r="K119">
-        <v>3.0986301369863014</v>
+        <v>3.117808219178082</v>
       </c>
       <c r="L119" t="s">
         <v>283</v>
@@ -7985,7 +7985,7 @@
         <v>0.23</v>
       </c>
       <c r="D120">
-        <v>3.8465753424657536</v>
+        <v>3.8657534246575347</v>
       </c>
       <c r="E120">
         <v>0.2</v>
@@ -8000,7 +8000,7 @@
         <v>285</v>
       </c>
       <c r="K120">
-        <v>3.8465753424657536</v>
+        <v>3.8657534246575342</v>
       </c>
       <c r="L120" t="s">
         <v>283</v>
@@ -8038,7 +8038,7 @@
         <v>0.36</v>
       </c>
       <c r="D121">
-        <v>6.002739726027397</v>
+        <v>6.021917808219178</v>
       </c>
       <c r="F121" t="s">
         <v>29</v>
@@ -8050,7 +8050,7 @@
         <v>282</v>
       </c>
       <c r="K121">
-        <v>6.857534246575343</v>
+        <v>6.876712328767123</v>
       </c>
       <c r="L121" t="s">
         <v>283</v>
@@ -8091,7 +8091,7 @@
         <v>0.3</v>
       </c>
       <c r="D122">
-        <v>3.041095890410959</v>
+        <v>3.0602739726027397</v>
       </c>
       <c r="E122">
         <v>4.4</v>
@@ -8106,7 +8106,7 @@
         <v>285</v>
       </c>
       <c r="K122">
-        <v>3.041095890410959</v>
+        <v>3.0602739726027397</v>
       </c>
       <c r="L122" t="s">
         <v>283</v>
@@ -8141,7 +8141,7 @@
         <v>0.15</v>
       </c>
       <c r="D123">
-        <v>4.419178082191781</v>
+        <v>4.438356164383562</v>
       </c>
       <c r="F123" t="s">
         <v>29</v>
@@ -8153,7 +8153,7 @@
         <v>67</v>
       </c>
       <c r="K123">
-        <v>13.673972602739726</v>
+        <v>13.693150684931506</v>
       </c>
       <c r="L123" t="s">
         <v>68</v>
@@ -8200,7 +8200,7 @@
         <v>0.15</v>
       </c>
       <c r="D124">
-        <v>4.419178082191781</v>
+        <v>4.438356164383562</v>
       </c>
       <c r="E124">
         <v>9.5</v>
@@ -8215,7 +8215,7 @@
         <v>67</v>
       </c>
       <c r="K124">
-        <v>13.673972602739726</v>
+        <v>13.693150684931506</v>
       </c>
       <c r="L124" t="s">
         <v>68</v>

</xml_diff>